<commit_message>
bug fix, add launch json
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C5364310\autoexcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA43A233-5EE0-411E-B3C0-EAD725BFBC59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05CF990-D8C2-4BF5-8F84-AD672E7DA06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{30301B15-6C27-4FB4-8355-8173C84860D2}"/>
   </bookViews>
@@ -36,12 +36,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>CS20260011979872 | CSM/FSM Configurable Workspace | ServiceNow</t>
+    <t>CS20260011864704 | CSM/FSM Configurable Workspace | ServiceNow</t>
   </si>
   <si>
-    <t>CS20260011978458 | CSM/FSM Configurable Workspace | ServiceNow</t>
+    <t>CS20260011683181 | CSM/FSM Configurable Workspace | ServiceNow</t>
+  </si>
+  <si>
+    <t>CS20260011844254 | CSM/FSM Configurable Workspace | ServiceNow</t>
+  </si>
+  <si>
+    <t>CS20260011875131 | CSM/FSM Configurable Workspace | ServiceNow</t>
   </si>
 </sst>
 </file>
@@ -424,8 +430,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74D8791D-B24E-43B7-9980-DE7F8FBADA0B}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="60.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -437,10 +446,28 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" r:id="rId1" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/53bd88fd2ff7b6541cead341bea4e345" xr:uid="{A2BEF53A-BB61-4046-9BAA-4333B238AFA4}"/>
-    <hyperlink ref="A2" r:id="rId2" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/ac92bfe5cff7fe1483c073903d851c70" xr:uid="{129B54D1-7CA0-498D-8D8E-2DAC1D4E8954}"/>
+    <hyperlink ref="A1" r:id="rId1" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/30db5581cfa37ed09912baeb4d851c7f" xr:uid="{0F8EAB46-0EAE-485A-9C23-0E8B8726C2BE}"/>
+    <hyperlink ref="A2" r:id="rId2" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/1286cfc93b83b6d4a6c6159e53e45a87" xr:uid="{9D12514A-B20B-4F7D-80CD-FC78FA34361D}"/>
+    <hyperlink ref="A3" r:id="rId3" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/f87592f32fd7f2501cead341bea4e3d9" xr:uid="{81AC37DC-3810-45EA-8EF5-A29165E637D9}"/>
+    <hyperlink ref="A4" r:id="rId4" display="https://itsm.services.sap/now/cwf/agent/record/sn_customerservice_case/6c840651cf67725423acfa713d851ceb" xr:uid="{9048E6C9-C75F-480A-9048-76D7EBC01E21}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>